<commit_message>
Fix ClinPGx --skip-download bug, update parser_review with latest counts
ClinPGx parse_data() now loads from cached JSON files when in-memory
lists are empty, fixing 0-row output with --skip-download. Updated
parser_review.xlsx with fresh pipeline counts: GWAS 760K, PubTator
69M+, ClinPGx restored to 454/378/1060.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parser_review.xlsx
+++ b/docs/parser_review.xlsx
@@ -608,7 +608,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Gene (193,687)</t>
+          <t>Gene (193,790)</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>genes.tsv: 193,791 lines</t>
+          <t>genes.tsv: 193,790 lines</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>disease_symptom: 3,358; disease_anatomy: 3,603; disease_disease: 544</t>
+          <t>disease_symptom: 3,357; disease_anatomy: 3,602; disease_disease: 543</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>symptom_nodes.tsv: 1,933 lines</t>
+          <t>symptom_nodes.tsv: 1,932 lines</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>pathways: 4,647; gene_pathway_rels: 187,248</t>
+          <t>pathways: 4,646; gene_pathway_rels: 187,247</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>disease_nodes: 12,013; disease_xrefs: 38,574</t>
+          <t>disease_nodes: 12,012; disease_xrefs: 38,573</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>drug_treats: 12,048; drug_palliates: 2,526</t>
+          <t>drug_treats: 11,805; drug_palliates: 2,505; pharm_class: 1,646; class_includes: 16,403</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Hetionet component parser</t>
+          <t>Loads CtD/CpD (drug treats/palliates disease), PharmClass nodes, and PCiC (pharmacologicClassIncludesCompound: 16,403 edges). Missing CbG (Compound-binds-Gene) from DrugCentral — but BindingDB covers CbG separately.</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>BP nodes: 24,548; MF nodes: 10,124; CC nodes: 4,070; gene-BP: 158,165; gene-MF: 106,410; gene-CC: 111,870</t>
+          <t>BP nodes: 24,547; MF nodes: 10,123; CC nodes: 4,069; gene-BP: 158,164; gene-MF: 106,409; gene-CC: 111,869</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>gene_disease_gwas.tsv: 44,191 lines</t>
+          <t>gene_disease_gwas.tsv: 760,270 lines</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Hetionet component parser</t>
+          <t>Full GWAS Catalog loaded. Maps GWAS traits to DOID diseases via 3-strategy DOID remap. 760,270 gene-disease associations (up from 90K with fresh download).</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>CuG: 33,025; CdG: 36,164; Gr&gt;G: 267,813</t>
+          <t>CuG: 33,024; CdG: 36,163; Gr&gt;G: 267,812</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>anatomy_nodes.tsv: 14,676 lines</t>
+          <t>anatomy_nodes.tsv: 14,675 lines</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>drug_binds_gene.tsv: 1,632,199 lines</t>
+          <t>drug_binds_gene.tsv: 23,954 lines</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Hetionet component parser</t>
+          <t>Human-only (Homo sapiens targets). Includes Ki/Kd/IC50 affinity data. 23,954 bindings after UniProt→Entrez mapping.</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>diseases: 901; gene_disease_assoc: 5,444</t>
+          <t>diseases: 900; gene_disease_assoc: 4,933</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>drugs.tsv: 19,843 lines</t>
+          <t>drugs.tsv: 19,842 lines</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>SE nodes: 5,735; CcSE edges: 153,664</t>
+          <t>SE nodes: 5,734; CcSE edges: 153,663</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>overexpresses: 3,201; underexpresses: 6,605,913</t>
+          <t>overexpresses: 3,200; underexpresses: 6,605,912</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>gene_covaries.tsv: 61,691 lines</t>
+          <t>gene_covaries.tsv: 61,690 lines</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -1993,7 +1993,7 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>gene_interacts.tsv: 147,165 lines</t>
+          <t>gene_interacts.tsv: 147,164 lines</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>trials: 8,329; conditions: 18,588; interventions: 12,348</t>
+          <t>trials: 14,856; conditions: 18,587; interventions: 12,347</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>annotations: 455; drug_labels: 379; variants: 1,061</t>
+          <t>annotations: 454; drug_labels: 378; variants: 1,060; gene_info: 17</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>CardioKB-specific new parser</t>
+          <t>CardioKB-specific. CVD pharmacogenomics (17 genes, 24 drugs) from ClinPGx REST API. Cache-loading fix applied for --skip-download support.</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>TFs: 368; TF-gene: 15,268</t>
+          <t>TFs: 367; TF-gene: 15,267</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>drugs: 173,501; pathways: 4,647; gene-pathway: 187,248</t>
+          <t>drugs: 173,500; pathways: 4,646; gene-pathway: 187,247</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>disease-disease: 2,154,921; gene-disease: 31,984,798</t>
+          <t>disease-disease: 9,367,474; gene-disease: 59,879,417</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>Hetionet component parser</t>
+          <t>Hetionet component parser. Massive literature mining: 69.2M+ edges total (59.9M gene-disease + 9.4M disease-disease).</t>
         </is>
       </c>
     </row>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>increases: 346,082; decreases: 330,935</t>
+          <t>increases: 346,081; decreases: 330,934</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -2606,22 +2606,22 @@
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>⏳ Pending</t>
+          <t>✅ Yes</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>(not yet loaded — no ontology configs)</t>
+          <t>Disease (enriched), Gene</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>(not yet loaded)</t>
+          <t>geneAssociatesWithDisease</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>(no TSVs generated)</t>
+          <t>cvd_gene_disease: 9,972; gene_disease_rels: 17,857; gene_phenotype: 18,953; cvd_genes: 1,653</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>AlzKB base parser</t>
+          <t>AlzKB base parser. Now fully working with OMIM_API_KEY. Generates CVD gene-disease relationships, gene phenotype maps.</t>
         </is>
       </c>
     </row>
@@ -2650,8 +2650,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A33:K33"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix Parser Type labels and column alignment in parser_review.xlsx
Corrected OMIM from 'AlzKB base parser' to 'CardioKB-specific new
parser'. Fixed several rows where Gaps/Mismatches text was written
to the Parser Type column. Audited all 29+8 rows for correct labels.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parser_review.xlsx
+++ b/docs/parser_review.xlsx
@@ -1013,12 +1013,12 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Loads CtD/CpD (drug treats/palliates disease) and PharmClass nodes. Missing CbG (Compound-binds-Gene) from DrugCentral — but BindingDB covers CbG separately. PCiC edges not loaded to Neo4j.</t>
+          <t>Loads CtD/CpD (drug treats/palliates disease), PharmClass nodes, and PCiC (pharmacologicClassIncludesCompound: 16,403 edges). Missing CbG (Compound-binds-Gene) from DrugCentral — but BindingDB covers CbG separately.</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Loads CtD/CpD (drug treats/palliates disease), PharmClass nodes, and PCiC (pharmacologicClassIncludesCompound: 16,403 edges). Missing CbG (Compound-binds-Gene) from DrugCentral — but BindingDB covers CbG separately.</t>
+          <t>Hetionet component parser</t>
         </is>
       </c>
     </row>
@@ -1123,12 +1123,12 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Full GWAS Catalog loaded. Maps GWAS traits to DOID diseases via mapped genes. No CVD-specific filtering (all traits).</t>
+          <t>Full GWAS Catalog loaded. Maps GWAS traits to DOID diseases via 3-strategy DOID remap. 760,270 gene-disease associations (up from 90K with fresh download).</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Full GWAS Catalog loaded. Maps GWAS traits to DOID diseases via 3-strategy DOID remap. 760,270 gene-disease associations (up from 90K with fresh download).</t>
+          <t>Hetionet component parser</t>
         </is>
       </c>
     </row>
@@ -1453,12 +1453,12 @@
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Human-only (Homo sapiens targets). Includes Ki/Kd/IC50 affinity data. 1.6M bindings vs Hetionet ~11K (much larger scope).</t>
+          <t>Human-only (Homo sapiens targets). Includes Ki/Kd/IC50 affinity data. 23,954 bindings after UniProt→Entrez mapping.</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Human-only (Homo sapiens targets). Includes Ki/Kd/IC50 affinity data. 23,954 bindings after UniProt→Entrez mapping.</t>
+          <t>Hetionet component parser</t>
         </is>
       </c>
     </row>
@@ -2289,12 +2289,12 @@
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>CardioKB-specific. CVD pharmacogenomics (17 genes, 24 drugs) from ClinPGx REST API.</t>
+          <t>CardioKB-specific. CVD pharmacogenomics (17 genes, 24 drugs) from ClinPGx REST API. Cache-loading fix applied for --skip-download support.</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>CardioKB-specific. CVD pharmacogenomics (17 genes, 24 drugs) from ClinPGx REST API. Cache-loading fix applied for --skip-download support.</t>
+          <t>CardioKB-specific new parser</t>
         </is>
       </c>
     </row>
@@ -2517,12 +2517,12 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Hetionet component parser. Massive literature mining: 34M+ edges total.</t>
+          <t>Hetionet component parser. Massive literature mining: 69.2M+ edges total (59.9M gene-disease + 9.4M disease-disease).</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>Hetionet component parser. Massive literature mining: 69.2M+ edges total (59.9M gene-disease + 9.4M disease-disease).</t>
+          <t>Hetionet component parser</t>
         </is>
       </c>
     </row>
@@ -2631,12 +2631,12 @@
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>AlzKB base parser. Parser code exists but no ontology configs; requires OMIM_API_KEY.</t>
+          <t>Now fully working with OMIM_API_KEY. Generates CVD gene-disease relationships, gene phenotype maps.</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>AlzKB base parser. Now fully working with OMIM_API_KEY. Generates CVD gene-disease relationships, gene phenotype maps.</t>
+          <t>CardioKB-specific new parser</t>
         </is>
       </c>
     </row>
@@ -2650,8 +2650,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A33:K33"/>
+    <mergeCell ref="A42:K42"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A42:K42"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix AOP-DB Parser Type to AlzKB base parser in parser_review.xlsx
AOP-DB is an AlzKB base parser (aopdb_parser.py), not CardioKB-specific.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parser_review.xlsx
+++ b/docs/parser_review.xlsx
@@ -853,7 +853,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>CardioKB-specific new parser</t>
+          <t>AlzKB base parser</t>
         </is>
       </c>
     </row>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>CardioKB-specific new parser</t>
+          <t>AlzKB base parser</t>
         </is>
       </c>
     </row>
@@ -2650,9 +2650,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A33:K33"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix minor column labels in parser_review.xlsx
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parser_review.xlsx
+++ b/docs/parser_review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nawaza/Desktop/Cardio-KB/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDFD59CE-354F-6D4A-83E1-5ABE6D11171D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5490B84-448E-8C49-8E12-6B8091144FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -698,12 +698,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF666666"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -853,19 +855,15 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -887,9 +885,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1209,34 +1211,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="22" t="s">
         <v>203</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="24" t="s">
         <v>202</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
     </row>
     <row r="3" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="8" t="s">
         <v>200</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -1263,7 +1265,7 @@
       <c r="J3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="K3" s="8" t="s">
         <v>201</v>
       </c>
     </row>
@@ -1271,7 +1273,7 @@
       <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="9" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -1306,7 +1308,7 @@
       <c r="A5" s="2">
         <v>2</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="18" t="s">
         <v>18</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1341,7 +1343,7 @@
       <c r="A6" s="2">
         <v>3</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="9" t="s">
         <v>26</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -1376,7 +1378,7 @@
       <c r="A7" s="2">
         <v>4</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="9" t="s">
         <v>34</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -1411,7 +1413,7 @@
       <c r="A8" s="2">
         <v>5</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="7" t="s">
         <v>197</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -1446,7 +1448,7 @@
       <c r="A9" s="2">
         <v>6</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="9" t="s">
         <v>45</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -1481,7 +1483,7 @@
       <c r="A10" s="2">
         <v>7</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="18" t="s">
         <v>51</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -1516,7 +1518,7 @@
       <c r="A11" s="2">
         <v>8</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="7" t="s">
         <v>56</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -1551,7 +1553,7 @@
       <c r="A12" s="2">
         <v>9</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="9" t="s">
         <v>63</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -1586,7 +1588,7 @@
       <c r="A13" s="2">
         <v>10</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="9" t="s">
         <v>70</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -1621,7 +1623,7 @@
       <c r="A14" s="2">
         <v>11</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="18" t="s">
         <v>76</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -1656,7 +1658,7 @@
       <c r="A15" s="2">
         <v>12</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="9" t="s">
         <v>81</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -1691,7 +1693,7 @@
       <c r="A16" s="2">
         <v>13</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="18" t="s">
         <v>87</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -1726,7 +1728,7 @@
       <c r="A17" s="2">
         <v>14</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="9" t="s">
         <v>92</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -1761,7 +1763,7 @@
       <c r="A18" s="2">
         <v>15</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="18" t="s">
         <v>97</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -1796,7 +1798,7 @@
       <c r="A19" s="2">
         <v>16</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="9" t="s">
         <v>100</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -1831,7 +1833,7 @@
       <c r="A20" s="2">
         <v>17</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="9" t="s">
         <v>106</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -1866,7 +1868,7 @@
       <c r="A21" s="2">
         <v>18</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="7" t="s">
         <v>111</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -1901,7 +1903,7 @@
       <c r="A22" s="2">
         <v>19</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="18" t="s">
         <v>117</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -1928,7 +1930,7 @@
       <c r="J22" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="K22" s="24" t="s">
+      <c r="K22" s="20" t="s">
         <v>216</v>
       </c>
     </row>
@@ -1936,7 +1938,7 @@
       <c r="A23" s="2">
         <v>20</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="18" t="s">
         <v>121</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -1963,7 +1965,7 @@
       <c r="J23" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="K23" s="24" t="s">
+      <c r="K23" s="20" t="s">
         <v>216</v>
       </c>
     </row>
@@ -1971,7 +1973,7 @@
       <c r="A24" s="2">
         <v>21</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="9" t="s">
         <v>124</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -2006,7 +2008,7 @@
       <c r="A25" s="2">
         <v>22</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="9" t="s">
         <v>131</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -2041,7 +2043,7 @@
       <c r="A26" s="2">
         <v>23</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="18" t="s">
         <v>136</v>
       </c>
       <c r="C26" s="2" t="s">
@@ -2076,7 +2078,7 @@
       <c r="A27" s="2">
         <v>24</v>
       </c>
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="18" t="s">
         <v>141</v>
       </c>
       <c r="C27" s="2" t="s">
@@ -2103,7 +2105,7 @@
       <c r="J27" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="K27" s="24" t="s">
+      <c r="K27" s="20" t="s">
         <v>216</v>
       </c>
     </row>
@@ -2111,7 +2113,7 @@
       <c r="A28" s="2">
         <v>25</v>
       </c>
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="16" t="s">
         <v>144</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -2146,7 +2148,7 @@
       <c r="A29" s="2">
         <v>26</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="16" t="s">
         <v>149</v>
       </c>
       <c r="C29" s="2" t="s">
@@ -2181,7 +2183,7 @@
       <c r="A30" s="2">
         <v>27</v>
       </c>
-      <c r="B30" s="20" t="s">
+      <c r="B30" s="16" t="s">
         <v>153</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -2216,7 +2218,7 @@
       <c r="A31" s="2">
         <v>28</v>
       </c>
-      <c r="B31" s="20" t="s">
+      <c r="B31" s="16" t="s">
         <v>157</v>
       </c>
       <c r="C31" s="2" t="s">
@@ -2251,7 +2253,7 @@
       <c r="A32" s="2">
         <v>29</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="18" t="s">
         <v>158</v>
       </c>
       <c r="C32" s="2" t="s">
@@ -2278,7 +2280,7 @@
       <c r="J32" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="K32" s="24" t="s">
+      <c r="K32" s="20" t="s">
         <v>216</v>
       </c>
     </row>
@@ -2286,7 +2288,7 @@
       <c r="A33" s="2">
         <v>30</v>
       </c>
-      <c r="B33" s="18" t="s">
+      <c r="B33" s="14" t="s">
         <v>161</v>
       </c>
       <c r="C33" s="2" t="s">
@@ -2321,7 +2323,7 @@
       <c r="A34" s="2">
         <v>31</v>
       </c>
-      <c r="B34" s="18" t="s">
+      <c r="B34" s="14" t="s">
         <v>169</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -2356,7 +2358,7 @@
       <c r="A35" s="2">
         <v>32</v>
       </c>
-      <c r="B35" s="14" t="s">
+      <c r="B35" s="10" t="s">
         <v>175</v>
       </c>
       <c r="C35" s="2" t="s">
@@ -2389,9 +2391,9 @@
     </row>
     <row r="36" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>35</v>
-      </c>
-      <c r="B36" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="10" t="s">
         <v>181</v>
       </c>
       <c r="C36" s="2" t="s">
@@ -2424,9 +2426,9 @@
     </row>
     <row r="37" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>36</v>
-      </c>
-      <c r="B37" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B37" s="10" t="s">
         <v>186</v>
       </c>
       <c r="C37" s="2" t="s">
@@ -2459,9 +2461,9 @@
     </row>
     <row r="38" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>37</v>
-      </c>
-      <c r="B38" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B38" s="14" t="s">
         <v>191</v>
       </c>
       <c r="C38" s="2" t="s">
@@ -2493,55 +2495,55 @@
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A39" s="8" t="s">
+      <c r="A39" s="25" t="s">
         <v>196</v>
       </c>
-      <c r="B39" s="7"/>
-      <c r="C39" s="7"/>
-      <c r="D39" s="7"/>
-      <c r="E39" s="7"/>
-      <c r="F39" s="7"/>
-      <c r="G39" s="7"/>
-      <c r="H39" s="7"/>
-      <c r="I39" s="7"/>
-      <c r="J39" s="7"/>
-      <c r="K39" s="7"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="23"/>
+      <c r="F39" s="23"/>
+      <c r="G39" s="23"/>
+      <c r="H39" s="23"/>
+      <c r="I39" s="23"/>
+      <c r="J39" s="23"/>
+      <c r="K39" s="23"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="F41" s="25"/>
+      <c r="F41" s="21"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B42" s="15"/>
+      <c r="B42" s="11"/>
       <c r="C42" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B43" s="16"/>
+      <c r="B43" s="12"/>
       <c r="C43" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B44" s="17"/>
+      <c r="B44" s="13"/>
       <c r="C44" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B45" s="19"/>
+      <c r="B45" s="15"/>
       <c r="C45" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B46" s="21"/>
+      <c r="B46" s="17"/>
       <c r="C46" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B47" s="23"/>
+      <c r="B47" s="19"/>
       <c r="C47" t="s">
         <v>215</v>
       </c>

</xml_diff>

<commit_message>
Fix STRING and OpenTargets rows in parser_review.xlsx
Unmerged corrupted row, rewrote both entries with proper cell data,
formatting, and green status fills matching existing table rows.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parser_review.xlsx
+++ b/docs/parser_review.xlsx
@@ -2656,110 +2656,110 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="20" t="n">
         <v>37</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="22" t="inlineStr">
         <is>
           <t>STRING</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>GiG (Gene-interacts-Gene protein interactions)</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>string_parser.py (STRINGParser)</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>(none — edge-only)</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>geneInteractsWithGene (228,193 edges)</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>gene_interactions: 228,193</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>STRING v12.0 human protein links, confidence &gt; 700. Maps ENSP IDs to gene symbols via aliases file. 228,193 high-confidence edges.</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>CardioKB-specific new parser</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="20" t="n">
         <v>38</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="22" t="inlineStr">
         <is>
           <t>Open Targets</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>GaD (Gene-associates-Disease)</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>opentargets_parser.py (OpenTargetsParser)</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>(none — edge-only)</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>geneAssociatesWithDisease (2,345,386 edges)</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>gene_disease: 2,345,386</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>Open Targets Platform 25.12 overall direct association scores (Parquet). EFO→DOID mapping via disease metadata dbXRefs. 2,345,386 gene-disease associations.</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>CardioKB-specific new parser</t>
         </is>
@@ -2772,7 +2772,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="F44" s="20" t="n"/>
     </row>
@@ -2835,7 +2834,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A40:K40"/>
+    <mergeCell ref="A42:K42"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add DrugAge, CellAge, AnAge, GenAge to parser_review.xlsx + fix README count
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parser_review.xlsx
+++ b/docs/parser_review.xlsx
@@ -606,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="28" min="1" max="1"/>
@@ -2949,66 +2949,295 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="27" t="inlineStr">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>DrugAge/CellAge</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>GaA (Gene-Aging associations)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>drugage_parser.py (DrugAgeParser)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>AgeingProperty (3)</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>associatedWithAging</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>gene_nodes, aging_property_nodes, gene_aging_association</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Gene-senescence effect associations from CellAge data. Creates AgeingProperty nodes (Induces/Inhibits/Unclear).</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Agent-generated parser</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>CellAge</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>G (Gene nodes)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>cellage_parser.py (CellAgeParser)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>(merge onto existing Gene nodes)</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(none - node enrichment only)</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>gene_nodes, gene_properties</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Cellular senescence gene list from CellAge. Node-only parser.</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Agent-generated parser</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>AnAge</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Sp (Species longevity)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>anage_parser.py (AnAgeParser)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>(none - node-only)</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>species_nodes</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Animal Ageing and Longevity Database. Species nodes with max lifespan, body mass, metabolic rate.</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Agent-generated parser</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>GenAge</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>G (Gene nodes)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>genage_parser.py (GenAgeParser)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>(merge onto existing Gene nodes)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>(none - node enrichment only)</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>gene_nodes</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Human ageing-associated genes from GenAge. Merges on geneSymbol.</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Agent-generated parser</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
         <is>
           <t>Legend — CardioKB Has It?: ✅ Yes | ⚠️ Partial | ❌ No | ⏳ Pending    |    Aligned?: ✅ Yes | ⚠️ Partial | ❌ No    |    Parser Type: AlzKB base parser | Hetionet component parser | CardioKB-specific new parser</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="F47" s="20" t="n"/>
-    </row>
-    <row r="48">
-      <c r="B48" s="10" t="n"/>
-      <c r="C48" t="inlineStr">
+    <row r="50"/>
+    <row r="51">
+      <c r="F51" s="20" t="n"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="10" t="n"/>
+      <c r="C52" t="inlineStr">
         <is>
           <t>Hetionet/Base component parser from AlzKB updater, exports nodes/edges same as Het.io</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="11" t="n"/>
-      <c r="C49" t="inlineStr">
+    <row r="53">
+      <c r="B53" s="11" t="n"/>
+      <c r="C53" t="inlineStr">
         <is>
           <t>Hetionet/Base component parser from AlzKB updater, partially works</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" s="12" t="n"/>
-      <c r="C50" t="inlineStr">
+    <row r="54">
+      <c r="B54" s="12" t="n"/>
+      <c r="C54" t="inlineStr">
         <is>
           <t>New parser added to AlzKB updater (not in OG Het.io)</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" s="14" t="n"/>
-      <c r="C51" t="inlineStr">
+    <row r="55">
+      <c r="B55" s="14" t="n"/>
+      <c r="C55" t="inlineStr">
         <is>
           <t>New parser added by Asma for CardioKB specifically</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="B52" s="16" t="n"/>
-      <c r="C52" t="inlineStr">
+    <row r="56">
+      <c r="B56" s="16" t="n"/>
+      <c r="C56" t="inlineStr">
         <is>
           <t>Hetionet_precomputed_parser</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="18" t="n"/>
-      <c r="C53" t="inlineStr">
+    <row r="57">
+      <c r="B57" s="18" t="n"/>
+      <c r="C57" t="inlineStr">
         <is>
           <t>In original Het.io, but not in AlzKB updater/CardioKB</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="B54" s="21" t="n"/>
-      <c r="C54" t="inlineStr">
+    <row r="58">
+      <c r="B58" s="21" t="n"/>
+      <c r="C58" t="inlineStr">
         <is>
           <t>Added from OG Het.io to complete pipeline (not yet in AlzKB updater)</t>
         </is>

</xml_diff>

<commit_message>
Update parser_review.xlsx with Neo4j-verified counts (46 cells updated)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parser_review.xlsx
+++ b/docs/parser_review.xlsx
@@ -733,7 +733,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Gene (193,790)</t>
+          <t>Gene (216,315)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>genes.tsv: 193,790 lines</t>
+          <t>genes.tsv: 216,315 lines</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>disease_symptom: 3,357; disease_anatomy: 3,602; disease_disease: 543</t>
+          <t>disease_symptom: 3,068; disease_anatomy: 3,602; disease_disease: 543</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Pathway (4,646)</t>
+          <t>Pathway (6,469)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>pathways: 4,646; gene_pathway_rels: 187,247</t>
+          <t>pathways: 6,469; gene_pathway_rels: 198,079 (each direction)</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Disease (12,012)</t>
+          <t>Disease (43,972)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>disease_nodes: 12,012; disease_xrefs: 38,573</t>
+          <t>disease_nodes: 43,972; disease_xrefs: 38,573</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">gene-disease associations: 44,394 </t>
+          <t>gene-disease associations: 20,563 (Neo4j verified)</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>drug_treats: 11,805; drug_palliates: 2,505; pharm_class: 1,646; class_includes: 16,403</t>
+          <t>drug_treats: 6,242; drug_palliates: 1,012; pharm_class: 1,646; class_includes: 16,403</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>BP nodes: 24,547; MF nodes: 10,123; CC nodes: 4,069; gene-BP: 158,164; gene-MF: 106,409; gene-CC: 111,869</t>
+          <t>BP nodes: 24,547; MF: 10,123; CC: 4,069; gene-BP: 135,351; gene-MF: 93,564; gene-CC: 93,792</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>gene_disease_gwas.tsv: 760,270 lines</t>
+          <t>gene_disease_gwas: 45,370 edges (Neo4j verified, after DOID remap)</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>pathway_nodes: 2,806; gene_pathway: 147,005</t>
+          <t>pathway_nodes: 2,806; gene_pathway: 96,394 (each direction)</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>CuG: 33,024; CdG: 36,163; Gr&gt;G: 267,812</t>
+          <t>CuG: 36,688; CdG: 40,895; Gr&gt;G: 279,578</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -1458,12 +1458,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">geneAssociatesWithBodyPart with source: "Jensen TISSUES"     </t>
+          <t>geneExpressedInBodyPart with source: "Jensen TISSUES"</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>gene-bodypart associations: 18,645</t>
+          <t>gene-tissue edges: 982,116 (Neo4j verified)</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>BodyPart (14,675)</t>
+          <t>BodyPart (14,937)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>anatomy_nodes.tsv: 14,675 lines</t>
+          <t>anatomy_nodes.tsv: 14,937 lines</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>pathway_nodes: 982; gene_pathway: 40,039</t>
+          <t>pathway_nodes: 982; gene_pathway: 46,271 (each direction)</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>drug_binds_gene.tsv: 23,954 lines</t>
+          <t>drug_binds_gene: 26,467 edges (Neo4j verified)</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>diseases: 900; gene_disease_assoc: 4,933</t>
+          <t>diseases: 900+; gene_disease_assoc: 23,704 (Neo4j verified)</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1753,17 +1753,17 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Drug (19,842)</t>
+          <t>Drug (46,142)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>drugBindsGene (19,047 edges)</t>
+          <t>drugBindsGene (19,085 edges)</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>drugs.tsv: 19,842; drug_binds_gene: 19,047</t>
+          <t>drugs: 46,142; drug_binds_gene: 19,085</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>SE nodes: 5,734; CcSE edges: 153,663</t>
+          <t>SE nodes: 5,734; CcSE edges: 148,518</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>overexpresses: 3,200; underexpresses: 6,605,912</t>
+          <t>overexpresses: 4,480; underexpresses: 7,211,055</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>gene_covaries.tsv: 61,690 lines</t>
+          <t>gene_covaries: 61,797 edges (Neo4j verified)</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>gene_interacts.tsv: 147,164 lines</t>
+          <t>gene_interacts: 136,283 edges (Neo4j, Hetionet source)</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>ClinicalTrial (14,856)</t>
+          <t>ClinicalTrial (576,334)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>trials: 14,856; conditions: 18,587; interventions: 12,347</t>
+          <t>trials: 576,334; STUDIES_CONDITION: 818,839; TESTS_INTERVENTION: 345,632</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>annotations: 454; drug_labels: 378; variants: 1,060; gene_info: 17</t>
+          <t>VARIANT_IN: 1,129; AFFECTS_RESPONSE_TO: 304; drugLabelAnnotatesGene: 506; drugLabelDescribesDrug: 360</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>TFs: 367; TF-gene: 15,267</t>
+          <t>TFs: 367; TF-gene: 15,092</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>disease-disease: 9,367,474; gene-disease: 59,879,417</t>
+          <t>disease-disease: 2,138,895; gene-disease: 14,908,646 (Neo4j verified)</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>increases: 346,081; decreases: 330,934</t>
+          <t>increases: 218,152; decreases: 213,587</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>cvd_gene_disease: 9,972; gene_disease_rels: 17,857; gene_phenotype: 18,953; cvd_genes: 1,653</t>
+          <t>gene_disease: 7,354 (Neo4j verified)</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>phenotype_nodes.tsv: 19,389; gene_phenotype_associations.tsv: 270,272</t>
+          <t>phenotype_nodes: 19,389; gene_phenotype: 303,817</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -2898,12 +2898,12 @@
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>geneInteractsWithGene (228,193 edges)</t>
+          <t>geneInteractsWithGene (229,485 edges)</t>
         </is>
       </c>
       <c r="H40" s="25" t="inlineStr">
         <is>
-          <t>gene_interactions: 228,193</t>
+          <t>gene_interactions: 229,485</t>
         </is>
       </c>
       <c r="I40" s="26" t="inlineStr">
@@ -2958,12 +2958,12 @@
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>geneAssociatesWithDisease (2,345,386 edges)</t>
+          <t>geneAssociatesWithDisease (2,388,123 edges)</t>
         </is>
       </c>
       <c r="H41" s="25" t="inlineStr">
         <is>
-          <t>gene_disease: 2,345,386</t>
+          <t>gene_disease: 2,388,123</t>
         </is>
       </c>
       <c r="I41" s="26" t="inlineStr">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="H42" s="31" t="inlineStr">
         <is>
-          <t>gene_nodes.tsv: 44,361</t>
+          <t>gene_nodes: 216,315 (enriched)</t>
         </is>
       </c>
       <c r="I42" s="26" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="G43" s="31" t="inlineStr">
         <is>
-          <t>geneInFamily / familyContainsGene (33,967 each)</t>
+          <t>geneInFamily / familyContainsGene (34,006 each)</t>
         </is>
       </c>
       <c r="H43" s="31" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="F44" s="31" t="inlineStr">
         <is>
-          <t>Variant (4,486,982)</t>
+          <t>Variant (4,488,042)</t>
         </is>
       </c>
       <c r="G44" s="31" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="H44" s="31" t="inlineStr">
         <is>
-          <t>variant_nodes: 4.5M; disease_variant: 5.7M; gene_variant: 4.5M</t>
+          <t>variants: 4,488,042; hasVariant: 4,439,480; variantInGene: 4,439,480; associatedWithVariant: 1,862,448; variantAssociatedWithDisease: 1,862,448</t>
         </is>
       </c>
       <c r="I44" s="26" t="inlineStr">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="F47" s="31" t="inlineStr">
         <is>
-          <t>Species</t>
+          <t>Species (8,032)</t>
         </is>
       </c>
       <c r="G47" s="31" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="H47" s="31" t="inlineStr">
         <is>
-          <t>species_nodes</t>
+          <t>species_nodes: 8,032</t>
         </is>
       </c>
       <c r="I47" s="26" t="inlineStr">

</xml_diff>

<commit_message>
Add relationship properties (expressionScore, zScore, morScore, confidence) + fresh Neo4j reload
- Added data_property_map to 6 ontology configs: Bgee (expressionScore),
  LINCS L1000 (zScore), DoRothEA (morScore + confidence)
- Clean Neo4j reload from TSVs: 4.9M nodes / 26.3M rels (36 sources, 0 failures)
- Updated README, CLAUDE.md, parser_review.xlsx with current graph stats

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parser_review.xlsx
+++ b/docs/parser_review.xlsx
@@ -733,7 +733,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Gene (216,315)</t>
+          <t>Gene (194,726)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>genes.tsv: 216,315 lines</t>
+          <t>genes.tsv: 194,726 lines</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>disease_symptom: 3,068; disease_anatomy: 3,602; disease_disease: 543</t>
+          <t>disease_symptom: 544; disease_anatomy: 615; disease_disease: 109</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>pathways: 6,469; gene_pathway_rels: 198,079 (each direction)</t>
+          <t>pathways: 6,469; gene_pathway_rels: 18,502 (each direction)</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Disease (43,972)</t>
+          <t>Disease (19,450)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>disease_nodes: 43,972; disease_xrefs: 38,573</t>
+          <t>disease_nodes: 19,450; disease_xrefs: 38,573</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -1098,12 +1098,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">geneAssociatesWithDisease with source: "Jensen DISEASES"     </t>
+          <t>geneAssociatesWithDisease with source: "Jensen DISEASES"</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>gene-disease associations: 20,563 (Neo4j verified)</t>
+          <t>gene-disease associations: 20,561 (Neo4j verified)</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>drug_treats: 6,242; drug_palliates: 1,012; pharm_class: 1,646; class_includes: 16,403</t>
+          <t>drug_treats: 1,326; drug_palliates: 292; pharm_class: 1,646; class_includes: 16,403</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>gene_disease_gwas: 45,370 edges (Neo4j verified, after DOID remap)</t>
+          <t>gene_disease_gwas: 45,529 edges (Neo4j verified, after DOID remap)</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>pathway_nodes: 2,806; gene_pathway: 96,394 (each direction)</t>
+          <t>pathway_nodes: 2,806; gene_pathway: 16,317 (each direction)</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>CuG: 36,688; CdG: 40,895; Gr&gt;G: 279,578</t>
+          <t>CuG: 4,686; CdG: 5,765; GrG: 6,262</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>gene-tissue edges: 982,116 (Neo4j verified)</t>
+          <t>gene-tissue edges: 982,039 (Neo4j verified)</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>pathway_nodes: 982; gene_pathway: 46,271 (each direction)</t>
+          <t>pathway_nodes: 982; gene_pathway: 8,564 (each direction)</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>drug_binds_gene: 26,467 edges (Neo4j verified)</t>
+          <t>drug_binds_gene: 4,205 edges (Neo4j verified)</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>diseases: 900+; gene_disease_assoc: 23,704 (Neo4j verified)</t>
+          <t>diseases: 900+; gene_disease_assoc: 20,046 (Neo4j verified)</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Drug (46,142)</t>
+          <t>Drug (41,566)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>drugs: 46,142; drug_binds_gene: 19,085</t>
+          <t>drugs: 41,566; drug_binds_gene: 19,085</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>overexpresses: 4,480; underexpresses: 7,211,055</t>
+          <t>overexpresses: 4,466; underexpresses: 5,334,316</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>gene_covaries: 61,797 edges (Neo4j verified)</t>
+          <t>gene_covaries: 127 edges (Neo4j verified)</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>gene_interacts: 136,283 edges (Neo4j, Hetionet source)</t>
+          <t>gene_interacts: 5,100 edges (Neo4j, Hetionet source)</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>ClinicalTrial (576,334)</t>
+          <t>ClinicalTrial (82,070)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>trials: 576,334; STUDIES_CONDITION: 818,839; TESTS_INTERVENTION: 345,632</t>
+          <t>trials: 82,070; STUDIES_CONDITION: 674; TESTS_INTERVENTION: 18,145</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>VARIANT_IN: 1,129; AFFECTS_RESPONSE_TO: 304; drugLabelAnnotatesGene: 506; drugLabelDescribesDrug: 360</t>
+          <t>VARIANT_IN: 1,103; AFFECTS_RESPONSE_TO: 304; drugLabelAnnotatesGene: 506; drugLabelDescribesDrug: 360</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>disease-disease: 2,138,895; gene-disease: 14,908,646 (Neo4j verified)</t>
+          <t>disease-disease: 2,138,895; gene-disease: 1,248,956 (Neo4j verified)</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>increases: 218,152; decreases: 213,587</t>
+          <t>increases: 218,140; decreases: 213,581</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>phenotype_nodes: 19,389; gene_phenotype: 303,817</t>
+          <t>phenotype_nodes: 19,389; gene_phenotype: 30,488</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -2898,12 +2898,12 @@
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>geneInteractsWithGene (229,485 edges)</t>
+          <t>geneInteractsWithGene (229,433 edges)</t>
         </is>
       </c>
       <c r="H40" s="25" t="inlineStr">
         <is>
-          <t>gene_interactions: 229,485</t>
+          <t>gene_interactions: 229,433</t>
         </is>
       </c>
       <c r="I40" s="26" t="inlineStr">
@@ -2958,12 +2958,12 @@
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>geneAssociatesWithDisease (2,388,123 edges)</t>
+          <t>geneAssociatesWithDisease (2,364,224 edges)</t>
         </is>
       </c>
       <c r="H41" s="25" t="inlineStr">
         <is>
-          <t>gene_disease: 2,388,123</t>
+          <t>gene_disease: 2,364,224</t>
         </is>
       </c>
       <c r="I41" s="26" t="inlineStr">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="H42" s="31" t="inlineStr">
         <is>
-          <t>gene_nodes: 216,315 (enriched)</t>
+          <t>gene_nodes: 194,726 (enriched)</t>
         </is>
       </c>
       <c r="I42" s="26" t="inlineStr">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="F47" s="31" t="inlineStr">
         <is>
-          <t>Species (8,032)</t>
+          <t>Species (4,645)</t>
         </is>
       </c>
       <c r="G47" s="31" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="H47" s="31" t="inlineStr">
         <is>
-          <t>species_nodes: 8,032</t>
+          <t>species_nodes: 4,645</t>
         </is>
       </c>
       <c r="I47" s="26" t="inlineStr">

</xml_diff>